<commit_message>
Automação: Bases de dados do GETS atualizadas
</commit_message>
<xml_diff>
--- a/planilhas_gets/03.Atividades/18.horasTrabalhadas_junho2026.xlsx
+++ b/planilhas_gets/03.Atividades/18.horasTrabalhadas_junho2026.xlsx
@@ -6,7 +6,7 @@
     <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="horasTrabalhadas20260629111004" r:id="rId3" sheetId="1"/>
+    <sheet name="horasTrabalhadas20260630091435" r:id="rId3" sheetId="1"/>
   </sheets>
 </workbook>
 </file>
@@ -96,8 +96,8 @@
       <c r="B4" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Data Início de 01/06/2026 até 29/06/2026
- Data Término de 01/06/2026 até 29/06/2026</t>
+ Data Início de 01/06/2026 até 30/06/2026
+ Data Término de 01/06/2026 até 30/06/2026</t>
         </is>
       </c>
     </row>

</xml_diff>